<commit_message>
replact text trong final_prompt
</commit_message>
<xml_diff>
--- a/data/video_scenario.xlsx
+++ b/data/video_scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\veo3\project\lion\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E3329E-56B7-440D-9A53-5736CDC6E0EB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888DFB82-9938-411A-B2AD-A807568E530E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
   <si>
     <t>template_key</t>
   </si>
@@ -32,30 +32,6 @@
     <t>note</t>
   </si>
   <si>
-    <t>Mẫu_Ảnh_Ngang_Anime</t>
-  </si>
-  <si>
-    <t>Anime style illustration of {0} wearing {1.0}, trending on pixiv, highly detailed --ar 16:9</t>
-  </si>
-  <si>
-    <t>Chỉ dùng {0} và {1}, bỏ qua ảnh tham chiếu</t>
-  </si>
-  <si>
-    <t>Mẫu_Ảnh_Ngang_Cinematic</t>
-  </si>
-  <si>
-    <t>"A cinematic scene of {1.0} fighting against {1.1} inside {2.0}, action: {0}"</t>
-  </si>
-  <si>
-    <t>Dùng đầy đủ cả 3 tham số đầu vào</t>
-  </si>
-  <si>
-    <t>NhanVat_and_Action</t>
-  </si>
-  <si>
-    <t>"{1.0}   {0}"</t>
-  </si>
-  <si>
     <t>scene_id</t>
   </si>
   <si>
@@ -80,26 +56,130 @@
     <t>file_name</t>
   </si>
   <si>
-    <t>scena_1</t>
-  </si>
-  <si>
-    <t>reading book</t>
-  </si>
-  <si>
-    <t>scena_2</t>
-  </si>
-  <si>
-    <t>close eyes</t>
-  </si>
-  <si>
-    <t>nvLion</t>
+    <t>vid_1</t>
+  </si>
+  <si>
+    <t>vid_2</t>
+  </si>
+  <si>
+    <t>vid_3</t>
+  </si>
+  <si>
+    <t>vid_4</t>
+  </si>
+  <si>
+    <t>vid_5</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>video_Anh_6x_4s</t>
+  </si>
+  <si>
+    <t>img_100</t>
+  </si>
+  <si>
+    <t>img_101</t>
+  </si>
+  <si>
+    <t>img_102</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create a continuous 5-second video that </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>pans and transitions sequentially through the 6-panel storyboard</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> layout of the selected image. The camera must start with a full-frame shot focusing exactly on Panel 1 (top-left). Then, the camera must </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>smoothly glide, pan, and transform forward through Panel 2, Panel 3, Panel 4, and Panel 5</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> in strict chronological order, creating a seamless frame-by-frame narrative flow. Finally, the video must </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>settle and resolve perfectly</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">on the content of Panel 6 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(bottom-right) as the cinematic ending. Ensure hyper-realistic wildlife documentary motion, smooth camera tracking, photorealistic textures, and zero abrupt cuts between the panels.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -111,6 +191,15 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -148,10 +237,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -455,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
@@ -466,68 +558,89 @@
     <col min="6" max="6" width="36.42578125" customWidth="1"/>
     <col min="7" max="7" width="33.7109375" customWidth="1"/>
     <col min="8" max="8" width="25.28515625" customWidth="1"/>
-    <col min="9" max="9" width="22.5703125" customWidth="1"/>
+    <col min="9" max="9" width="38.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
+        <v>17</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="2" t="s">
         <v>19</v>
       </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="E7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -536,7 +649,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -554,37 +667,21 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Run video success, get asset_name
</commit_message>
<xml_diff>
--- a/data/video_scenario.xlsx
+++ b/data/video_scenario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\veo3\project\lion\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888DFB82-9938-411A-B2AD-A807568E530E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F29653D9-D896-4B98-8C8A-D0D37C4812FB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>template_key</t>
   </si>
@@ -65,29 +65,23 @@
     <t>vid_3</t>
   </si>
   <si>
-    <t>vid_4</t>
-  </si>
-  <si>
-    <t>vid_5</t>
-  </si>
-  <si>
     <t>Normal</t>
   </si>
   <si>
     <t>video_Anh_6x_4s</t>
   </si>
   <si>
-    <t>img_100</t>
-  </si>
-  <si>
-    <t>img_101</t>
-  </si>
-  <si>
-    <t>img_102</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Create a continuous 5-second video that </t>
+    <t>On the open grasslands, everything appears calm.</t>
+  </si>
+  <si>
+    <t>A small herd of antelope grazes peacefully.</t>
+  </si>
+  <si>
+    <t>A close-up shot focused on thick</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Create a continuous -second video that </t>
     </r>
     <r>
       <rPr>
@@ -173,6 +167,21 @@
       </rPr>
       <t>(bottom-right) as the cinematic ending. Ensure hyper-realistic wildlife documentary motion, smooth camera tracking, photorealistic textures, and zero abrupt cuts between the panels.</t>
     </r>
+  </si>
+  <si>
+    <t>Create a seamless, continuous 4-second video that morphs and transitions smoothly between the two selected images, starting with the first image and ending perfectly on the second image. The text "{0}" must be clearly printed as a static, clean, white minimalist subtitle at the bottom center of the screen throughout the entire video to distinguish this scene. Through highly fluid animation, the elements must transform continuously forward without any cuts. Ensure hyper-realistic textures, consistent cinematic wildlife style, and extremely smooth motion interpolation, while keeping the text label completely rigid and crisp.</t>
+  </si>
+  <si>
+    <t>Only_title_4s</t>
+  </si>
+  <si>
+    <t>mage_1, mage_2</t>
+  </si>
+  <si>
+    <t>mage_2, mage_3</t>
+  </si>
+  <si>
+    <t>mage_3, mage_4</t>
   </si>
 </sst>
 </file>
@@ -590,26 +599,32 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -617,26 +632,13 @@
         <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>21</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -649,7 +651,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -669,15 +671,23 @@
     </row>
     <row r="2" spans="1:3" ht="119.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>